<commit_message>
initial move of world/base region logic from code to conversion script
</commit_message>
<xml_diff>
--- a/Conversion Script/Set_filter_file.xlsx
+++ b/Conversion Script/Set_filter_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nim\Documents\GENeSYS_MOD.data\Conversion Script\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E54952-63F6-448C-BC8A-6573727563BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D940B5C4-03A3-4096-A661-E967C6DCD76E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{0B764928-35F8-4A30-ADCD-C0369050184D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{0B764928-35F8-4A30-ADCD-C0369050184D}"/>
   </bookViews>
   <sheets>
     <sheet name="Region_selection" sheetId="1" r:id="rId1"/>
@@ -1259,12 +1259,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A667788-FC3C-4C43-9E46-ED47A2AEE749}">
   <dimension ref="A1:C55"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>217</v>
       </c>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>221</v>
       </c>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1298,7 +1298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1306,7 +1306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1330,7 +1330,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1338,7 +1338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -1346,7 +1346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1354,7 +1354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1362,7 +1362,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -1394,7 +1394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -1402,7 +1402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -1410,7 +1410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -1434,7 +1434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1442,7 +1442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -1450,7 +1450,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -1466,7 +1466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -1490,7 +1490,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1498,7 +1498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -1514,7 +1514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -1522,7 +1522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -1530,7 +1530,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -1554,7 +1554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>222</v>
       </c>
@@ -1570,7 +1570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>223</v>
       </c>
@@ -1578,7 +1578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>224</v>
       </c>
@@ -1586,7 +1586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>225</v>
       </c>
@@ -1594,7 +1594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>226</v>
       </c>
@@ -1602,7 +1602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>227</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>228</v>
       </c>
@@ -1618,7 +1618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>229</v>
       </c>
@@ -1626,7 +1626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>230</v>
       </c>
@@ -1634,7 +1634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>231</v>
       </c>
@@ -1642,7 +1642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>232</v>
       </c>
@@ -1650,7 +1650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>233</v>
       </c>
@@ -1658,7 +1658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>234</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>235</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>236</v>
       </c>
@@ -1682,7 +1682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>237</v>
       </c>
@@ -1690,7 +1690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>238</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>239</v>
       </c>
@@ -1714,12 +1714,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C5D2E10-6D88-4A1E-9C1A-BD9E15FD6A9D}">
   <dimension ref="A1:B148"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>146</v>
       </c>
@@ -1727,7 +1727,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>37</v>
       </c>
@@ -1735,7 +1735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -1743,7 +1743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -1751,7 +1751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -1775,7 +1775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>44</v>
       </c>
@@ -1791,7 +1791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>45</v>
       </c>
@@ -1799,7 +1799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>46</v>
       </c>
@@ -1807,7 +1807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -1815,7 +1815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>48</v>
       </c>
@@ -1823,7 +1823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>49</v>
       </c>
@@ -1831,7 +1831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>50</v>
       </c>
@@ -1839,7 +1839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>51</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>52</v>
       </c>
@@ -1855,7 +1855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>53</v>
       </c>
@@ -1863,7 +1863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>54</v>
       </c>
@@ -1871,7 +1871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>55</v>
       </c>
@@ -1879,7 +1879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>56</v>
       </c>
@@ -1887,7 +1887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>57</v>
       </c>
@@ -1895,7 +1895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>58</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>277</v>
       </c>
@@ -1911,7 +1911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>59</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>60</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>61</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>62</v>
       </c>
@@ -1943,7 +1943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>63</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>64</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>65</v>
       </c>
@@ -1967,7 +1967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>66</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>67</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>68</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>69</v>
       </c>
@@ -1999,7 +1999,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>70</v>
       </c>
@@ -2007,7 +2007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>71</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>244</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>245</v>
       </c>
@@ -2031,7 +2031,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>246</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>247</v>
       </c>
@@ -2047,7 +2047,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>248</v>
       </c>
@@ -2055,7 +2055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>249</v>
       </c>
@@ -2063,7 +2063,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>250</v>
       </c>
@@ -2071,7 +2071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>251</v>
       </c>
@@ -2079,7 +2079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>252</v>
       </c>
@@ -2087,7 +2087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>253</v>
       </c>
@@ -2095,7 +2095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>254</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>255</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>73</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>74</v>
       </c>
@@ -2127,7 +2127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>75</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>76</v>
       </c>
@@ -2143,7 +2143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>77</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>78</v>
       </c>
@@ -2159,7 +2159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>79</v>
       </c>
@@ -2167,7 +2167,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>80</v>
       </c>
@@ -2175,7 +2175,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>81</v>
       </c>
@@ -2183,7 +2183,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>72</v>
       </c>
@@ -2191,7 +2191,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>82</v>
       </c>
@@ -2199,7 +2199,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>83</v>
       </c>
@@ -2207,7 +2207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>84</v>
       </c>
@@ -2215,7 +2215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>85</v>
       </c>
@@ -2223,7 +2223,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>86</v>
       </c>
@@ -2231,7 +2231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>87</v>
       </c>
@@ -2239,7 +2239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>88</v>
       </c>
@@ -2247,7 +2247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>89</v>
       </c>
@@ -2255,7 +2255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>90</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>91</v>
       </c>
@@ -2271,7 +2271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>93</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>94</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>92</v>
       </c>
@@ -2295,7 +2295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>95</v>
       </c>
@@ -2303,7 +2303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>96</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>97</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>98</v>
       </c>
@@ -2327,7 +2327,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>99</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>100</v>
       </c>
@@ -2343,7 +2343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>101</v>
       </c>
@@ -2351,7 +2351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>102</v>
       </c>
@@ -2359,7 +2359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>103</v>
       </c>
@@ -2367,7 +2367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>104</v>
       </c>
@@ -2375,7 +2375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>262</v>
       </c>
@@ -2383,7 +2383,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>105</v>
       </c>
@@ -2391,7 +2391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>108</v>
       </c>
@@ -2399,7 +2399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>106</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>107</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>263</v>
       </c>
@@ -2423,7 +2423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>109</v>
       </c>
@@ -2431,7 +2431,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>280</v>
       </c>
@@ -2439,7 +2439,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>281</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>110</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>264</v>
       </c>
@@ -2463,7 +2463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>111</v>
       </c>
@@ -2471,7 +2471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>265</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>266</v>
       </c>
@@ -2487,7 +2487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>267</v>
       </c>
@@ -2495,7 +2495,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>268</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>269</v>
       </c>
@@ -2511,7 +2511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>270</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>271</v>
       </c>
@@ -2527,7 +2527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>272</v>
       </c>
@@ -2535,7 +2535,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>273</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>274</v>
       </c>
@@ -2551,7 +2551,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>275</v>
       </c>
@@ -2559,7 +2559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>276</v>
       </c>
@@ -2567,7 +2567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>112</v>
       </c>
@@ -2575,7 +2575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>113</v>
       </c>
@@ -2583,7 +2583,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>114</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>115</v>
       </c>
@@ -2599,7 +2599,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>116</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>117</v>
       </c>
@@ -2615,7 +2615,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
         <v>118</v>
       </c>
@@ -2623,7 +2623,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
         <v>119</v>
       </c>
@@ -2631,7 +2631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
         <v>120</v>
       </c>
@@ -2639,7 +2639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
         <v>121</v>
       </c>
@@ -2647,7 +2647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>256</v>
       </c>
@@ -2655,7 +2655,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>122</v>
       </c>
@@ -2663,7 +2663,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>123</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>124</v>
       </c>
@@ -2679,7 +2679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>257</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>125</v>
       </c>
@@ -2695,7 +2695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>126</v>
       </c>
@@ -2703,7 +2703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>258</v>
       </c>
@@ -2711,7 +2711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>259</v>
       </c>
@@ -2719,7 +2719,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>260</v>
       </c>
@@ -2727,7 +2727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>261</v>
       </c>
@@ -2735,7 +2735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>240</v>
       </c>
@@ -2743,7 +2743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>243</v>
       </c>
@@ -2751,7 +2751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>127</v>
       </c>
@@ -2759,7 +2759,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
         <v>128</v>
       </c>
@@ -2767,7 +2767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
         <v>129</v>
       </c>
@@ -2775,7 +2775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>130</v>
       </c>
@@ -2783,7 +2783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>131</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
         <v>132</v>
       </c>
@@ -2799,7 +2799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
         <v>133</v>
       </c>
@@ -2807,7 +2807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>134</v>
       </c>
@@ -2815,7 +2815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>241</v>
       </c>
@@ -2823,7 +2823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>135</v>
       </c>
@@ -2831,7 +2831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>136</v>
       </c>
@@ -2839,7 +2839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>242</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>137</v>
       </c>
@@ -2855,7 +2855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>138</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>139</v>
       </c>
@@ -2871,7 +2871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
         <v>140</v>
       </c>
@@ -2879,7 +2879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>141</v>
       </c>
@@ -2887,7 +2887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>142</v>
       </c>
@@ -2895,7 +2895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>143</v>
       </c>
@@ -2921,12 +2921,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B82051EE-CB34-4773-B6E9-985CB3357CE5}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>181</v>
       </c>
@@ -2934,7 +2934,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>182</v>
       </c>
@@ -2942,7 +2942,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>183</v>
       </c>
@@ -2950,7 +2950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>184</v>
       </c>
@@ -2958,7 +2958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>185</v>
       </c>
@@ -2966,7 +2966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>278</v>
       </c>
@@ -2974,7 +2974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>186</v>
       </c>
@@ -2982,7 +2982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>187</v>
       </c>
@@ -2990,7 +2990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>188</v>
       </c>
@@ -3006,12 +3006,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C7942D6-5BBA-4326-BEB2-07D45E712A14}">
   <dimension ref="A1:B31"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>149</v>
       </c>
@@ -3019,7 +3019,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>150</v>
       </c>
@@ -3027,7 +3027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>151</v>
       </c>
@@ -3035,7 +3035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>152</v>
       </c>
@@ -3043,7 +3043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>153</v>
       </c>
@@ -3051,7 +3051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>154</v>
       </c>
@@ -3059,7 +3059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>155</v>
       </c>
@@ -3067,7 +3067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>156</v>
       </c>
@@ -3075,7 +3075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>157</v>
       </c>
@@ -3083,7 +3083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>158</v>
       </c>
@@ -3091,7 +3091,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>159</v>
       </c>
@@ -3099,7 +3099,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>160</v>
       </c>
@@ -3107,7 +3107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>161</v>
       </c>
@@ -3115,7 +3115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>162</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>163</v>
       </c>
@@ -3131,7 +3131,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>279</v>
       </c>
@@ -3139,7 +3139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>164</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>165</v>
       </c>
@@ -3155,7 +3155,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>166</v>
       </c>
@@ -3163,7 +3163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>167</v>
       </c>
@@ -3171,7 +3171,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>168</v>
       </c>
@@ -3179,7 +3179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>169</v>
       </c>
@@ -3187,7 +3187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>170</v>
       </c>
@@ -3195,7 +3195,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>171</v>
       </c>
@@ -3203,7 +3203,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>172</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>173</v>
       </c>
@@ -3219,7 +3219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>168</v>
       </c>
@@ -3227,7 +3227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>174</v>
       </c>
@@ -3235,7 +3235,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>175</v>
       </c>
@@ -3243,7 +3243,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>176</v>
       </c>
@@ -3251,7 +3251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>177</v>
       </c>
@@ -3275,9 +3275,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A951553-3765-459F-BC61-BDBD26E96FE5}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>179</v>
       </c>
@@ -3285,7 +3285,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3293,7 +3293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3301,7 +3301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3309,7 +3309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3325,9 +3325,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{755CD133-F9DD-44F8-9E58-F17622E607C5}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>144</v>
       </c>
@@ -3335,7 +3335,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>145</v>
       </c>
@@ -3351,9 +3351,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C358E473-EC7A-41C0-8602-044D340269A5}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>220</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>190</v>
       </c>
@@ -3369,7 +3369,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>191</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>192</v>
       </c>
@@ -3385,7 +3385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>193</v>
       </c>
@@ -3393,7 +3393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>194</v>
       </c>
@@ -3401,7 +3401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>195</v>
       </c>
@@ -3409,7 +3409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>196</v>
       </c>
@@ -3417,7 +3417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>197</v>
       </c>
@@ -3425,7 +3425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>198</v>
       </c>
@@ -3433,7 +3433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>199</v>
       </c>
@@ -3441,7 +3441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>200</v>
       </c>
@@ -3449,7 +3449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>201</v>
       </c>
@@ -3457,7 +3457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>202</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>203</v>
       </c>
@@ -3473,7 +3473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>204</v>
       </c>
@@ -3481,7 +3481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>205</v>
       </c>
@@ -3489,7 +3489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>206</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>207</v>
       </c>
@@ -3513,9 +3513,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96D5B3E0-498C-4AB7-BB30-7BCE295E19AC}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>219</v>
       </c>
@@ -3523,7 +3523,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>158</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>209</v>
       </c>
@@ -3539,7 +3539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>210</v>
       </c>
@@ -3547,7 +3547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>211</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>212</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>213</v>
       </c>
@@ -3571,7 +3571,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>214</v>
       </c>
@@ -3579,7 +3579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>215</v>
       </c>
@@ -3595,9 +3595,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5D817F8-1014-4E28-A827-54661E8BA006}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>218</v>
       </c>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2015</v>
       </c>
@@ -3614,7 +3614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2018</v>
       </c>
@@ -3622,7 +3622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2019</v>
       </c>
@@ -3630,7 +3630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2020</v>
       </c>
@@ -3638,7 +3638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2025</v>
       </c>
@@ -3646,7 +3646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2030</v>
       </c>
@@ -3654,7 +3654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2035</v>
       </c>
@@ -3662,7 +3662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2040</v>
       </c>
@@ -3670,7 +3670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2045</v>
       </c>
@@ -3678,7 +3678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2050</v>
       </c>

</xml_diff>

<commit_message>
updates regarding hydrogen (SMR) and syngas
</commit_message>
<xml_diff>
--- a/Conversion Script/Set_filter_file.xlsx
+++ b/Conversion Script/Set_filter_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jb\GENeSYS_MOD.data\Conversion Script\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nim\Documents\GENeSYS_MOD.data\Conversion Script\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{805B50C3-8859-4C20-88E2-044E3AFC19E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F5188F-4A0D-4D24-9D2A-C2439A3B6139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="6" activeTab="9" xr2:uid="{0B764928-35F8-4A30-ADCD-C0369050184D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" activeTab="3" xr2:uid="{0B764928-35F8-4A30-ADCD-C0369050184D}"/>
   </bookViews>
   <sheets>
     <sheet name="Region_selection" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
     <definedName name="Fuels">#REF!</definedName>
     <definedName name="Technologies">#REF!:B</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1216,7 +1216,7 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1232,9 +1232,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1272,7 +1272,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1378,7 +1378,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1529,12 +1529,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A667788-FC3C-4C43-9E46-ED47A2AEE749}">
   <dimension ref="A1:C55"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>203</v>
       </c>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>207</v>
       </c>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1560,7 +1560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1568,7 +1568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1576,7 +1576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1584,7 +1584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1592,7 +1592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1608,7 +1608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -1616,7 +1616,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1624,7 +1624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -1640,7 +1640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1648,7 +1648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -1664,7 +1664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -1680,7 +1680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -1688,7 +1688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -1704,7 +1704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -1720,7 +1720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -1728,7 +1728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -1736,7 +1736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -1744,7 +1744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -1752,7 +1752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -1760,7 +1760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1768,7 +1768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -1776,7 +1776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -1792,7 +1792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -1808,7 +1808,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -1816,7 +1816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -1832,7 +1832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>208</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>209</v>
       </c>
@@ -1848,7 +1848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>210</v>
       </c>
@@ -1856,7 +1856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>211</v>
       </c>
@@ -1864,7 +1864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>212</v>
       </c>
@@ -1872,7 +1872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>213</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>214</v>
       </c>
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>215</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>216</v>
       </c>
@@ -1904,7 +1904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>217</v>
       </c>
@@ -1912,7 +1912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>218</v>
       </c>
@@ -1920,7 +1920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>219</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>220</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>221</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>222</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>223</v>
       </c>
@@ -1960,7 +1960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>224</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>225</v>
       </c>
@@ -1984,9 +1984,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{738B5DF0-4614-4AAA-8D30-A109FA3624F2}">
   <dimension ref="A1:C75"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>294</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>297</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>298</v>
       </c>
@@ -2019,7 +2019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>299</v>
       </c>
@@ -2030,7 +2030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>300</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>301</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>302</v>
       </c>
@@ -2063,7 +2063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>303</v>
       </c>
@@ -2074,7 +2074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>304</v>
       </c>
@@ -2085,7 +2085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>305</v>
       </c>
@@ -2096,7 +2096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>306</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>307</v>
       </c>
@@ -2118,7 +2118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>308</v>
       </c>
@@ -2129,7 +2129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>309</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>310</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>311</v>
       </c>
@@ -2162,7 +2162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>312</v>
       </c>
@@ -2173,7 +2173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>313</v>
       </c>
@@ -2184,7 +2184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>314</v>
       </c>
@@ -2195,7 +2195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>315</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>316</v>
       </c>
@@ -2217,7 +2217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>317</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>318</v>
       </c>
@@ -2239,7 +2239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>319</v>
       </c>
@@ -2250,7 +2250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>320</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>321</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>322</v>
       </c>
@@ -2283,7 +2283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>323</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>324</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>325</v>
       </c>
@@ -2316,7 +2316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>326</v>
       </c>
@@ -2327,7 +2327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>327</v>
       </c>
@@ -2338,7 +2338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>328</v>
       </c>
@@ -2349,7 +2349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>329</v>
       </c>
@@ -2360,7 +2360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>330</v>
       </c>
@@ -2371,7 +2371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>331</v>
       </c>
@@ -2382,7 +2382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>332</v>
       </c>
@@ -2393,7 +2393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>333</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>334</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>335</v>
       </c>
@@ -2426,7 +2426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>336</v>
       </c>
@@ -2437,7 +2437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>337</v>
       </c>
@@ -2448,7 +2448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>338</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>339</v>
       </c>
@@ -2470,7 +2470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>340</v>
       </c>
@@ -2481,7 +2481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>341</v>
       </c>
@@ -2492,7 +2492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>342</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>343</v>
       </c>
@@ -2514,7 +2514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>344</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>345</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>346</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>347</v>
       </c>
@@ -2558,7 +2558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>348</v>
       </c>
@@ -2569,7 +2569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>349</v>
       </c>
@@ -2580,7 +2580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>350</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>351</v>
       </c>
@@ -2602,7 +2602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>352</v>
       </c>
@@ -2613,7 +2613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>353</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>354</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>355</v>
       </c>
@@ -2646,7 +2646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>356</v>
       </c>
@@ -2657,7 +2657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>357</v>
       </c>
@@ -2668,7 +2668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>358</v>
       </c>
@@ -2679,7 +2679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>359</v>
       </c>
@@ -2690,7 +2690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>360</v>
       </c>
@@ -2701,7 +2701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>361</v>
       </c>
@@ -2712,7 +2712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>362</v>
       </c>
@@ -2723,7 +2723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>363</v>
       </c>
@@ -2734,7 +2734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>364</v>
       </c>
@@ -2745,7 +2745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>365</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>366</v>
       </c>
@@ -2767,7 +2767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>367</v>
       </c>
@@ -2778,7 +2778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>368</v>
       </c>
@@ -2789,7 +2789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>369</v>
       </c>
@@ -2800,7 +2800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>370</v>
       </c>
@@ -2819,12 +2819,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C5D2E10-6D88-4A1E-9C1A-BD9E15FD6A9D}">
   <dimension ref="A1:B154"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>133</v>
       </c>
@@ -2832,7 +2832,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>37</v>
       </c>
@@ -2840,7 +2840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -2848,7 +2848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -2856,7 +2856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -2872,7 +2872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -2880,7 +2880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -2888,7 +2888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>44</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>45</v>
       </c>
@@ -2904,7 +2904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>46</v>
       </c>
@@ -2912,7 +2912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -2920,7 +2920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>48</v>
       </c>
@@ -2928,7 +2928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>49</v>
       </c>
@@ -2936,7 +2936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>50</v>
       </c>
@@ -2944,7 +2944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>51</v>
       </c>
@@ -2952,7 +2952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>52</v>
       </c>
@@ -2960,7 +2960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>289</v>
       </c>
@@ -2968,7 +2968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>53</v>
       </c>
@@ -2976,7 +2976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -2984,7 +2984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>55</v>
       </c>
@@ -2992,7 +2992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>56</v>
       </c>
@@ -3000,7 +3000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>57</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>276</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>277</v>
       </c>
@@ -3024,7 +3024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>278</v>
       </c>
@@ -3032,7 +3032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>58</v>
       </c>
@@ -3040,7 +3040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -3048,7 +3048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>60</v>
       </c>
@@ -3056,7 +3056,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>61</v>
       </c>
@@ -3064,7 +3064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>62</v>
       </c>
@@ -3072,7 +3072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>63</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>64</v>
       </c>
@@ -3088,7 +3088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>65</v>
       </c>
@@ -3096,7 +3096,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>66</v>
       </c>
@@ -3104,7 +3104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>67</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>68</v>
       </c>
@@ -3120,7 +3120,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>69</v>
       </c>
@@ -3128,7 +3128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>70</v>
       </c>
@@ -3136,7 +3136,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>230</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>231</v>
       </c>
@@ -3152,7 +3152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>232</v>
       </c>
@@ -3160,7 +3160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>233</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>234</v>
       </c>
@@ -3176,7 +3176,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>235</v>
       </c>
@@ -3184,7 +3184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>236</v>
       </c>
@@ -3192,7 +3192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>237</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>238</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>239</v>
       </c>
@@ -3216,7 +3216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>240</v>
       </c>
@@ -3224,7 +3224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>282</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>283</v>
       </c>
@@ -3240,7 +3240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>284</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>285</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>286</v>
       </c>
@@ -3264,7 +3264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>71</v>
       </c>
@@ -3272,7 +3272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>72</v>
       </c>
@@ -3280,7 +3280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>73</v>
       </c>
@@ -3288,7 +3288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>74</v>
       </c>
@@ -3296,7 +3296,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>75</v>
       </c>
@@ -3304,7 +3304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>76</v>
       </c>
@@ -3312,7 +3312,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>77</v>
       </c>
@@ -3320,7 +3320,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>78</v>
       </c>
@@ -3328,7 +3328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>79</v>
       </c>
@@ -3336,7 +3336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>80</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>81</v>
       </c>
@@ -3352,7 +3352,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>82</v>
       </c>
@@ -3360,7 +3360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>83</v>
       </c>
@@ -3368,7 +3368,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>84</v>
       </c>
@@ -3376,7 +3376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>85</v>
       </c>
@@ -3384,7 +3384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>86</v>
       </c>
@@ -3392,7 +3392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>87</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>266</v>
       </c>
@@ -3408,7 +3408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>267</v>
       </c>
@@ -3416,7 +3416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>268</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>269</v>
       </c>
@@ -3432,7 +3432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>270</v>
       </c>
@@ -3440,7 +3440,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>271</v>
       </c>
@@ -3448,7 +3448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>272</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>273</v>
       </c>
@@ -3464,7 +3464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>274</v>
       </c>
@@ -3472,7 +3472,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>88</v>
       </c>
@@ -3480,7 +3480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>89</v>
       </c>
@@ -3488,7 +3488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>90</v>
       </c>
@@ -3496,7 +3496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>91</v>
       </c>
@@ -3504,7 +3504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>92</v>
       </c>
@@ -3512,7 +3512,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>93</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>247</v>
       </c>
@@ -3528,7 +3528,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>94</v>
       </c>
@@ -3536,7 +3536,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>97</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>95</v>
       </c>
@@ -3552,7 +3552,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>96</v>
       </c>
@@ -3560,7 +3560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>248</v>
       </c>
@@ -3568,7 +3568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>98</v>
       </c>
@@ -3576,7 +3576,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>263</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>264</v>
       </c>
@@ -3592,7 +3592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>99</v>
       </c>
@@ -3600,7 +3600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>249</v>
       </c>
@@ -3608,7 +3608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>100</v>
       </c>
@@ -3616,7 +3616,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>250</v>
       </c>
@@ -3624,7 +3624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>251</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>252</v>
       </c>
@@ -3640,7 +3640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>253</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>254</v>
       </c>
@@ -3656,7 +3656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>255</v>
       </c>
@@ -3664,7 +3664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>256</v>
       </c>
@@ -3672,7 +3672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>257</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>258</v>
       </c>
@@ -3688,7 +3688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>259</v>
       </c>
@@ -3696,7 +3696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>260</v>
       </c>
@@ -3704,7 +3704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>261</v>
       </c>
@@ -3712,7 +3712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>101</v>
       </c>
@@ -3720,7 +3720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>102</v>
       </c>
@@ -3728,7 +3728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>103</v>
       </c>
@@ -3736,7 +3736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>104</v>
       </c>
@@ -3744,7 +3744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>105</v>
       </c>
@@ -3752,7 +3752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>106</v>
       </c>
@@ -3760,7 +3760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>107</v>
       </c>
@@ -3768,7 +3768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>108</v>
       </c>
@@ -3776,7 +3776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>109</v>
       </c>
@@ -3784,7 +3784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>110</v>
       </c>
@@ -3792,7 +3792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>241</v>
       </c>
@@ -3800,7 +3800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>111</v>
       </c>
@@ -3808,7 +3808,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>112</v>
       </c>
@@ -3816,7 +3816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>113</v>
       </c>
@@ -3824,7 +3824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>242</v>
       </c>
@@ -3832,7 +3832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>114</v>
       </c>
@@ -3840,7 +3840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>115</v>
       </c>
@@ -3848,7 +3848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>243</v>
       </c>
@@ -3856,7 +3856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>244</v>
       </c>
@@ -3864,7 +3864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>245</v>
       </c>
@@ -3872,7 +3872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>290</v>
       </c>
@@ -3880,7 +3880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>246</v>
       </c>
@@ -3888,7 +3888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>226</v>
       </c>
@@ -3896,7 +3896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>229</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>116</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>292</v>
       </c>
@@ -3920,7 +3920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>117</v>
       </c>
@@ -3928,7 +3928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>118</v>
       </c>
@@ -3936,7 +3936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>275</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>119</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>120</v>
       </c>
@@ -3960,7 +3960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>121</v>
       </c>
@@ -3968,7 +3968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>227</v>
       </c>
@@ -3976,7 +3976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>122</v>
       </c>
@@ -3984,7 +3984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>123</v>
       </c>
@@ -3992,7 +3992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>228</v>
       </c>
@@ -4000,23 +4000,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>124</v>
       </c>
       <c r="B148">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>125</v>
       </c>
       <c r="B149">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>126</v>
       </c>
@@ -4024,7 +4024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>127</v>
       </c>
@@ -4032,7 +4032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>128</v>
       </c>
@@ -4040,7 +4040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>129</v>
       </c>
@@ -4048,7 +4048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>130</v>
       </c>
@@ -4074,12 +4074,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B82051EE-CB34-4773-B6E9-985CB3357CE5}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>168</v>
       </c>
@@ -4087,7 +4087,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>171</v>
       </c>
@@ -4095,7 +4095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>172</v>
       </c>
@@ -4103,7 +4103,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>173</v>
       </c>
@@ -4111,7 +4111,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>170</v>
       </c>
@@ -4119,7 +4119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>174</v>
       </c>
@@ -4127,7 +4127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>279</v>
       </c>
@@ -4135,7 +4135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>281</v>
       </c>
@@ -4143,7 +4143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>280</v>
       </c>
@@ -4151,7 +4151,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>169</v>
       </c>
@@ -4172,12 +4172,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C7942D6-5BBA-4326-BEB2-07D45E712A14}">
   <dimension ref="A1:B35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>136</v>
       </c>
@@ -4185,7 +4185,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>160</v>
       </c>
@@ -4193,7 +4193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>137</v>
       </c>
@@ -4201,7 +4201,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>138</v>
       </c>
@@ -4209,7 +4209,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>154</v>
       </c>
@@ -4217,7 +4217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>139</v>
       </c>
@@ -4225,7 +4225,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>161</v>
       </c>
@@ -4233,23 +4233,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>162</v>
       </c>
       <c r="B8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>163</v>
       </c>
       <c r="B9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>149</v>
       </c>
@@ -4257,7 +4257,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>142</v>
       </c>
@@ -4265,7 +4265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>150</v>
       </c>
@@ -4273,7 +4273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>141</v>
       </c>
@@ -4281,7 +4281,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>265</v>
       </c>
@@ -4289,7 +4289,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>140</v>
       </c>
@@ -4297,7 +4297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>262</v>
       </c>
@@ -4305,7 +4305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>164</v>
       </c>
@@ -4313,7 +4313,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>153</v>
       </c>
@@ -4321,7 +4321,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>151</v>
       </c>
@@ -4329,7 +4329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>152</v>
       </c>
@@ -4337,7 +4337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>287</v>
       </c>
@@ -4345,7 +4345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>288</v>
       </c>
@@ -4353,7 +4353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>157</v>
       </c>
@@ -4361,7 +4361,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>159</v>
       </c>
@@ -4369,7 +4369,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>148</v>
       </c>
@@ -4377,7 +4377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>156</v>
       </c>
@@ -4385,7 +4385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>158</v>
       </c>
@@ -4393,7 +4393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>146</v>
       </c>
@@ -4401,7 +4401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>147</v>
       </c>
@@ -4409,7 +4409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>143</v>
       </c>
@@ -4417,7 +4417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>144</v>
       </c>
@@ -4425,7 +4425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>145</v>
       </c>
@@ -4433,7 +4433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>155</v>
       </c>
@@ -4441,7 +4441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>155</v>
       </c>
@@ -4449,7 +4449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>291</v>
       </c>
@@ -4476,9 +4476,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A951553-3765-459F-BC61-BDBD26E96FE5}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>166</v>
       </c>
@@ -4486,7 +4486,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4494,7 +4494,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -4502,7 +4502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -4510,7 +4510,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -4518,7 +4518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -4526,7 +4526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -4542,9 +4542,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{755CD133-F9DD-44F8-9E58-F17622E607C5}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>131</v>
       </c>
@@ -4552,7 +4552,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>132</v>
       </c>
@@ -4568,9 +4568,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C358E473-EC7A-41C0-8602-044D340269A5}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>206</v>
       </c>
@@ -4578,7 +4578,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>176</v>
       </c>
@@ -4586,7 +4586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>177</v>
       </c>
@@ -4594,7 +4594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>178</v>
       </c>
@@ -4602,7 +4602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>179</v>
       </c>
@@ -4610,7 +4610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>180</v>
       </c>
@@ -4618,7 +4618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>181</v>
       </c>
@@ -4626,7 +4626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>182</v>
       </c>
@@ -4634,7 +4634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>183</v>
       </c>
@@ -4642,7 +4642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>184</v>
       </c>
@@ -4650,7 +4650,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>185</v>
       </c>
@@ -4658,7 +4658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>186</v>
       </c>
@@ -4666,7 +4666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>187</v>
       </c>
@@ -4674,7 +4674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>188</v>
       </c>
@@ -4682,7 +4682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>189</v>
       </c>
@@ -4690,7 +4690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>190</v>
       </c>
@@ -4698,7 +4698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>191</v>
       </c>
@@ -4706,7 +4706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>192</v>
       </c>
@@ -4714,7 +4714,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>193</v>
       </c>
@@ -4730,9 +4730,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96D5B3E0-498C-4AB7-BB30-7BCE295E19AC}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>205</v>
       </c>
@@ -4740,7 +4740,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>145</v>
       </c>
@@ -4748,7 +4748,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>195</v>
       </c>
@@ -4756,7 +4756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>196</v>
       </c>
@@ -4764,7 +4764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>197</v>
       </c>
@@ -4772,7 +4772,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>198</v>
       </c>
@@ -4780,7 +4780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>199</v>
       </c>
@@ -4788,7 +4788,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>200</v>
       </c>
@@ -4796,7 +4796,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>201</v>
       </c>
@@ -4804,7 +4804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>293</v>
       </c>
@@ -4820,9 +4820,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5D817F8-1014-4E28-A827-54661E8BA006}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>204</v>
       </c>
@@ -4831,7 +4831,7 @@
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2015</v>
       </c>
@@ -4839,7 +4839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2018</v>
       </c>
@@ -4847,7 +4847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2019</v>
       </c>
@@ -4855,7 +4855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2020</v>
       </c>
@@ -4863,7 +4863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2021</v>
       </c>
@@ -4871,7 +4871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2025</v>
       </c>
@@ -4879,7 +4879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2030</v>
       </c>
@@ -4887,7 +4887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2035</v>
       </c>
@@ -4895,7 +4895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2040</v>
       </c>
@@ -4903,7 +4903,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2045</v>
       </c>
@@ -4911,7 +4911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2050</v>
       </c>
@@ -4919,7 +4919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2055</v>
       </c>
@@ -4927,7 +4927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2060</v>
       </c>

</xml_diff>

<commit_message>
added reviewer comments for PR to main (see PR of gms repo)
</commit_message>
<xml_diff>
--- a/Conversion Script/Set_filter_file.xlsx
+++ b/Conversion Script/Set_filter_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nim\Documents\GENeSYS_MOD.data\Conversion Script\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F5188F-4A0D-4D24-9D2A-C2439A3B6139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAE00CAE-335C-46CA-8505-4B74AC058949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" activeTab="3" xr2:uid="{0B764928-35F8-4A30-ADCD-C0369050184D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{0B764928-35F8-4A30-ADCD-C0369050184D}"/>
   </bookViews>
   <sheets>
     <sheet name="Region_selection" sheetId="1" r:id="rId1"/>
@@ -4238,7 +4238,7 @@
         <v>162</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -4246,7 +4246,7 @@
         <v>163</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>